<commit_message>
Add Week05 hands-on (DB + Flask dashboard) and organize Week04 files
- Week05: DB concept, AI-driven SQL queries, Flask web dashboard exercises
  with step-by-step guides (step0~3), answer scripts, and create_db.py
- Move root-level PDF/PPTX/ZIP into week04-hands-on/
- Add week04 automation scripts (expense_report, merge_sales, verify_all)
- Add week04 CLAUDE.md harness and askill.md verification spec

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/week04-hands-on/data/[재경]경비정리_202603_v1.xlsx
+++ b/week04-hands-on/data/[재경]경비정리_202603_v1.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,17 +29,41 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+        <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,15 +71,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,6 +465,13 @@
   </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -452,78 +501,78 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>92000</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>270000</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="E2" s="3" t="n">
         <v>362000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>106000</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>95000</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="E3" s="3" t="n">
         <v>201000</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>관리팀</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>146000</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>146000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="B5" s="1" t="n">
+      <c r="B5" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="5" t="n">
         <v>344000</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="5" t="n">
         <v>365000</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="E5" s="5" t="n">
         <v>709000</v>
       </c>
     </row>
@@ -540,6 +589,15 @@
   </sheetPr>
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -579,489 +637,489 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>15000</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-03-03</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>식대</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>32000</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>28000</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>개인카드</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>개인카드 - 정산대상</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2026-03-07</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>관리팀</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>사무용품</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>45000</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="G5" s="2" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-03-09</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>식대</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>18000</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" s="2" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>2026-03-11</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>접대비</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="7" t="n">
         <v>120000</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>특별경비</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>※ 증빙 첨부 필수</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>관리팀</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>12000</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>개인카드</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>개인카드 - 정산대상</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-03-15</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>25000</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="G9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>2026-03-17</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>식대</t>
         </is>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="3" t="n">
         <v>35000</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="G10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>관리팀</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>사무용품</t>
         </is>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>67000</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="G11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>접대비</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="7" t="n">
         <v>95000</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>개인카드</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>특별경비</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>※ 팀장 사전승인</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>2026-03-23</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n">
+      <c r="D13" s="3" t="n">
         <v>14000</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-03-25</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>관리팀</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>식대</t>
         </is>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <v>22000</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D15" s="3" t="n">
         <v>31000</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>개인카드</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>일반경비</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>개인카드 - 정산대상</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>2026-03-29</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>접대비</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="7" t="n">
         <v>150000</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>법인카드</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>특별경비</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>※ 증빙 첨부 필수</t>
         </is>
@@ -1080,6 +1138,13 @@
   </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1109,100 +1174,100 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-03-05</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>영업1팀</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>28000</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>미정산</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-03-13</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>관리팀</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" s="3" t="n">
         <v>12000</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>미정산</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-03-21</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>접대비</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>95000</v>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>미정산</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2026-03-27</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>영업2팀</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>교통비</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>31000</v>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>미정산</t>
         </is>

</xml_diff>